<commit_message>
Update documentation and workbook summary
</commit_message>
<xml_diff>
--- a/excel/Credit_Structuring_Cash_Flow_Engine.xlsx
+++ b/excel/Credit_Structuring_Cash_Flow_Engine.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="R4941f29694584b15"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Inputs" sheetId="2" r:id="R99c7ca103cd64202"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cash Flows" sheetId="3" r:id="Rf68015d63cbe4dc6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sensitivities" sheetId="4" r:id="R2a5568f5977f4fb1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Checks" sheetId="5" r:id="Rad53861216be4129"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources &amp; Notes" sheetId="6" r:id="R9de9acb2316c495e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="R32240797a8db4ef4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Inputs" sheetId="2" r:id="Rc9409e58b25b4ad5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cash Flows" sheetId="3" r:id="R33ee2df3b3194550"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sensitivities" sheetId="4" r:id="R692a1a0761fd482b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Checks" sheetId="5" r:id="R410c8f2c3e324851"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources &amp; Notes" sheetId="6" r:id="Ra11cf1c103b1467d"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -839,7 +839,7 @@
         <x:color rgb="FF006100"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFE2F0D9"/>
         </x:patternFill>
       </x:fill>
@@ -850,7 +850,7 @@
         <x:color rgb="FF9C0006"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFCE4D6"/>
         </x:patternFill>
       </x:fill>
@@ -861,7 +861,7 @@
         <x:color rgb="FF006100"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFE2F0D9"/>
         </x:patternFill>
       </x:fill>
@@ -872,7 +872,7 @@
         <x:color rgb="FF9C6500"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFF2CC"/>
         </x:patternFill>
       </x:fill>
@@ -883,7 +883,7 @@
         <x:color rgb="FF9C0006"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFCE4D6"/>
         </x:patternFill>
       </x:fill>
@@ -894,7 +894,7 @@
         <x:color rgb="FF006100"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFE2F0D9"/>
         </x:patternFill>
       </x:fill>
@@ -905,7 +905,7 @@
         <x:color rgb="FF9C6500"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFF2CC"/>
         </x:patternFill>
       </x:fill>
@@ -916,7 +916,7 @@
         <x:color rgb="FF9C0006"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFCE4D6"/>
         </x:patternFill>
       </x:fill>
@@ -927,7 +927,7 @@
         <x:color rgb="FF006100"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFE2F0D9"/>
         </x:patternFill>
       </x:fill>
@@ -938,7 +938,7 @@
         <x:color rgb="FF9C6500"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFF2CC"/>
         </x:patternFill>
       </x:fill>
@@ -949,7 +949,7 @@
         <x:color rgb="FF9C0006"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFCE4D6"/>
         </x:patternFill>
       </x:fill>
@@ -1492,18 +1492,10 @@
       </x:c>
       <x:c r="C16" s="111"/>
       <x:c r="D16" s="111"/>
-      <x:c r="E16" s="120" t="str">
-        <x:v>Boundary</x:v>
-      </x:c>
-      <x:c r="F16" s="121" t="str">
-        <x:v>Indicative educational model</x:v>
-      </x:c>
-      <x:c r="G16" s="121" t="str">
-        <x:v>Not an executable quote</x:v>
-      </x:c>
-      <x:c r="H16" s="122" t="str">
-        <x:v>Not investment advice</x:v>
-      </x:c>
+      <x:c r="E16"/>
+      <x:c r="F16"/>
+      <x:c r="G16"/>
+      <x:c r="H16"/>
     </x:row>
     <x:row r="17">
       <x:c r="A17" s="111" t="str">
@@ -1568,17 +1560,17 @@
       <x:c r="D21" s="10" t="str">
         <x:v>VALUATION COMPONENTS</x:v>
       </x:c>
-      <x:c r="E21" s="10" t="str">
-        <x:v>REVIEWER ROUTE</x:v>
-      </x:c>
-      <x:c r="F21" s="10" t="str">
-        <x:v>REVIEWER ROUTE</x:v>
-      </x:c>
-      <x:c r="G21" s="10" t="str">
-        <x:v>REVIEWER ROUTE</x:v>
-      </x:c>
-      <x:c r="H21" s="10" t="str">
-        <x:v>REVIEWER ROUTE</x:v>
+      <x:c r="E21" t="str">
+        <x:v>Start here: Summary → Inputs → Cash Flows → Sensitivities → Checks</x:v>
+      </x:c>
+      <x:c r="F21" t="str">
+        <x:v>Start here: Summary → Inputs → Cash Flows → Sensitivities → Checks</x:v>
+      </x:c>
+      <x:c r="G21" t="str">
+        <x:v>Start here: Summary → Inputs → Cash Flows → Sensitivities → Checks</x:v>
+      </x:c>
+      <x:c r="H21" t="str">
+        <x:v>Start here: Summary → Inputs → Cash Flows → Sensitivities → Checks</x:v>
       </x:c>
     </x:row>
     <x:row r="22">
@@ -1591,18 +1583,10 @@
       </x:c>
       <x:c r="C22" s="111"/>
       <x:c r="D22" s="111"/>
-      <x:c r="E22" s="50" t="str">
-        <x:v>Step</x:v>
-      </x:c>
-      <x:c r="F22" s="51" t="str">
-        <x:v>Action</x:v>
-      </x:c>
-      <x:c r="G22" s="51" t="str">
-        <x:v>Evidence</x:v>
-      </x:c>
-      <x:c r="H22" s="52" t="str">
-        <x:v>Approx. time</x:v>
-      </x:c>
+      <x:c r="E22"/>
+      <x:c r="F22"/>
+      <x:c r="G22"/>
+      <x:c r="H22"/>
     </x:row>
     <x:row r="23">
       <x:c r="A23" s="111" t="str">
@@ -1614,18 +1598,10 @@
       </x:c>
       <x:c r="C23" s="111"/>
       <x:c r="D23" s="111"/>
-      <x:c r="E23" s="115" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="F23" s="116" t="str">
-        <x:v>Read the Summary</x:v>
-      </x:c>
-      <x:c r="G23" s="116" t="str">
-        <x:v>Product map and economics</x:v>
-      </x:c>
-      <x:c r="H23" s="117" t="str">
-        <x:v>45 sec</x:v>
-      </x:c>
+      <x:c r="E23"/>
+      <x:c r="F23"/>
+      <x:c r="G23"/>
+      <x:c r="H23"/>
     </x:row>
     <x:row r="24">
       <x:c r="A24" s="111" t="str">
@@ -1637,18 +1613,10 @@
       </x:c>
       <x:c r="C24" s="111"/>
       <x:c r="D24" s="111"/>
-      <x:c r="E24" s="115" t="n">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="F24" s="116" t="str">
-        <x:v>Change Inputs B6, B16 or B17</x:v>
-      </x:c>
-      <x:c r="G24" s="116" t="str">
-        <x:v>Reusable product template</x:v>
-      </x:c>
-      <x:c r="H24" s="117" t="str">
-        <x:v>60 sec</x:v>
-      </x:c>
+      <x:c r="E24"/>
+      <x:c r="F24"/>
+      <x:c r="G24"/>
+      <x:c r="H24"/>
     </x:row>
     <x:row r="25">
       <x:c r="A25" s="111" t="str">
@@ -1660,18 +1628,10 @@
       </x:c>
       <x:c r="C25" s="111"/>
       <x:c r="D25" s="111"/>
-      <x:c r="E25" s="115" t="n">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="F25" s="116" t="str">
-        <x:v>Inspect Cash Flows</x:v>
-      </x:c>
-      <x:c r="G25" s="116" t="str">
-        <x:v>Default and survival mechanics</x:v>
-      </x:c>
-      <x:c r="H25" s="117" t="str">
-        <x:v>75 sec</x:v>
-      </x:c>
+      <x:c r="E25"/>
+      <x:c r="F25"/>
+      <x:c r="G25"/>
+      <x:c r="H25"/>
     </x:row>
     <x:row r="26">
       <x:c r="A26" s="111" t="str">
@@ -1683,18 +1643,10 @@
       </x:c>
       <x:c r="C26" s="111"/>
       <x:c r="D26" s="111"/>
-      <x:c r="E26" s="115" t="n">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="F26" s="116" t="str">
-        <x:v>Review Sensitivities</x:v>
-      </x:c>
-      <x:c r="G26" s="116" t="str">
-        <x:v>Spread and recovery risk</x:v>
-      </x:c>
-      <x:c r="H26" s="117" t="str">
-        <x:v>60 sec</x:v>
-      </x:c>
+      <x:c r="E26"/>
+      <x:c r="F26"/>
+      <x:c r="G26"/>
+      <x:c r="H26"/>
     </x:row>
     <x:row r="27">
       <x:c r="A27" s="111" t="str">
@@ -1706,18 +1658,10 @@
       </x:c>
       <x:c r="C27" s="111"/>
       <x:c r="D27" s="111"/>
-      <x:c r="E27" s="115" t="n">
-        <x:v>5</x:v>
-      </x:c>
-      <x:c r="F27" s="116" t="str">
-        <x:v>Confirm Checks</x:v>
-      </x:c>
-      <x:c r="G27" s="116" t="str">
-        <x:v>Controls and Python cross-check</x:v>
-      </x:c>
-      <x:c r="H27" s="117" t="str">
-        <x:v>60 sec</x:v>
-      </x:c>
+      <x:c r="E27"/>
+      <x:c r="F27"/>
+      <x:c r="G27"/>
+      <x:c r="H27"/>
     </x:row>
     <x:row r="28">
       <x:c r="A28" s="111" t="str">
@@ -1729,10 +1673,10 @@
       </x:c>
       <x:c r="C28" s="111"/>
       <x:c r="D28" s="111"/>
-      <x:c r="E28" s="115"/>
-      <x:c r="F28" s="116"/>
-      <x:c r="G28" s="116"/>
-      <x:c r="H28" s="117"/>
+      <x:c r="E28"/>
+      <x:c r="F28"/>
+      <x:c r="G28"/>
+      <x:c r="H28"/>
     </x:row>
     <x:row r="29">
       <x:c r="A29" s="111" t="str">
@@ -1744,18 +1688,10 @@
       </x:c>
       <x:c r="C29" s="111"/>
       <x:c r="D29" s="111"/>
-      <x:c r="E29" s="115" t="str">
-        <x:v>Production extensions</x:v>
-      </x:c>
-      <x:c r="F29" s="116" t="str">
-        <x:v>Market curves, ISDA settlement, counterparty risk and booking integration</x:v>
-      </x:c>
-      <x:c r="G29" s="116" t="str">
-        <x:v>Explicitly excluded</x:v>
-      </x:c>
-      <x:c r="H29" s="117" t="str">
-        <x:v>Discussion</x:v>
-      </x:c>
+      <x:c r="E29"/>
+      <x:c r="F29"/>
+      <x:c r="G29"/>
+      <x:c r="H29"/>
     </x:row>
     <x:row r="30">
       <x:c r="A30" s="111" t="str">
@@ -1767,18 +1703,10 @@
       </x:c>
       <x:c r="C30" s="111"/>
       <x:c r="D30" s="111"/>
-      <x:c r="E30" s="120" t="str">
-        <x:v>Source of truth</x:v>
-      </x:c>
-      <x:c r="F30" s="121" t="str">
-        <x:v>Python engine with an independent formula mirror in Excel</x:v>
-      </x:c>
-      <x:c r="G30" s="121" t="str">
-        <x:v>Tests plus workbook checks</x:v>
-      </x:c>
-      <x:c r="H30" s="122" t="str">
-        <x:v>Discussion</x:v>
-      </x:c>
+      <x:c r="E30"/>
+      <x:c r="F30"/>
+      <x:c r="G30"/>
+      <x:c r="H30"/>
     </x:row>
     <x:row r="31">
       <x:c r="A31" s="111" t="str">
@@ -2556,7 +2484,7 @@
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb18c27470f854409"/>
+  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfca11bac8ea0484a"/>
 </x:worksheet>
 </file>
 

</xml_diff>